<commit_message>
feat(test): offline pytest harness, auth fixtures, and Excel trackers (P1-3)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +45,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00137333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="005F6368"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -94,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -102,6 +107,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -816,6 +822,90 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SEC-201</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>P1-3</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Test JWT Token Replay / Cross-Environment Guard</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>CWE-347</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Test tokens signed with static test key could be replayed against non-test instances if secrets matched.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Production runtime enforces unique production JWT secret via Pydantic model validator, rendering test tokens invalid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SEC-202</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>P1-3</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Ephemeral Database and Checkpoint Isolation</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>CWE-212</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Test suites writing to persistent SQLite files risk leaking sensitive test fixtures onto disk.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>conftest.py enforces in-memory SQLite and checkpoints (:memory:) guaranteeing zero residual disk state.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(infra): Makefile, .env.example, deployment tests, and Phase 1 completion (P1-4)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -906,6 +906,90 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>SEC-301</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>P1-4</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Environment Secret Exposure Verification in Template</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>CWE-200</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Template files checked into source control risk leaking developer secrets or live API keys.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Verified .env.example contains safe placeholders only; automated test_no_committed_env_file gates CI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SEC-302</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>P1-4</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Makefile Shell Injection and Parameter Safety</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>CWE-78</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Makefile recipes running external commands could suffer command injection if unquoted variables were used.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>POSIX-compliant parameter expansion with safe fallback defaults (${BASE_URL:-http://localhost:8000}).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(db): SQLAlchemy entities and category enum (P2-1)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Vulnerabilities" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vulnerabilities" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -990,6 +990,90 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SEC-401</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>P2-1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SQL Injection Mitigation via Declarative Mapped Types</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CWE-89</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Improperly sanitized user inputs in SQL statements could allow SQL injection.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SQLAlchemy 2.0 type-annotated mapped_column with parameterized queries and strict input typing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SEC-402</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>P2-1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Relational Cascade Integrity and Audit Immutability</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CWE-404</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Cascading deletes could inadvertently purge security audit logs or leave orphaned child records.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Configured ondelete=CASCADE on transient children and isolated AuditLog without foreign key cascade, guaranteeing immutable audit trails.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(db): Postgres schema, RLS policies, and migrations (P2-2)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1074,6 +1074,90 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SEC-501</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>P2-2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Service Role Key Isolation and RLS Anon Containment</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CWE-285</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Service role key could be leaked to client bundles or anon role granted unintended table access.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Strict client key isolation (anon key only on client) and RLS denies anon access across all tables except published articles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SEC-502</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>P2-2</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Trigger Function Search Path Manipulation</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CWE-426</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Functions executing without schema qualification could suffer search_path hijack.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>set_updated_at plpgsql function explicitly references NOW() and operates safely within trigger scope.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(db): async database core and repository layer (P2-3)
- Implement backend/app/core/database.py async engine and session lifecycle
- Implement generic BaseRepository with standardized async CRUD operations
- Implement CustomerRepository and WorkspaceRepository for customer 360 profiling
- Implement TicketRepository and TicketMessageRepository with atomic creation and chronological ordering
- Implement ApprovalRepository for human-in-the-loop approval workflows
- Implement CustomerMemoryRepository for recent customer notes recall
- Add 11 unit/integration tests in tests/unit/test_repositories.py (TC-061 to TC-071)
- Remediate SEC-601 (credential masking) and SEC-602 (parameterized query generation)
- Update TEST_CASES.xlsx, SECURITY_VULNERABILITIES.xlsx, TASKS.md, and MEMORY.md
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vulnerabilities" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Vulnerabilities" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1158,6 +1158,90 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SEC-601</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>P2-3</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Database Connection String and Credential Sanitization</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CWE-209</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Database connection URLs with embedded credentials could be exposed in debug logs or uncaught exception traces.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Database engine configured with echo=False; JSON logging formatter automatically masks sensitive fields (password, secret, token, key).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SEC-602</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>P2-3</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Parameterized ORM Filtering and Attribute Access Control</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CWE-89</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Dynamic filter values or malicious search strings could lead to SQL injection or unauthorized attribute access.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Repository queries strictly utilize SQLAlchemy 2.0 type-safe expressions with parameterized query generation; verified via SQL injection test.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(demo): sample data fixtures and demo bootstrap service (P2-4)
- Create sample_data datasets: customers.json (8 customers across 4 plans), subscriptions.json, workspaces.json, products.json, incidents.json, previous_resolutions.json, tickets.json (CD-1001 to CD-1013)
- Create 15 knowledge base articles with YAML frontmatter covering all 10 canonical categories
- Create database/seed.sql containing PostgreSQL INSERT fixtures
- Implement backend/app/services/seed_service.py for idempotent demo bootstrapping
- Integrate demo table creation and bootstrap into backend/app/main.py lifespan
- Add 8 unit/integration tests in tests/unit/test_seed_service.py (TC-072 to TC-079)
- Document and remediate SEC-701 and SEC-702
- Update TEST_CASES.xlsx, SECURITY_VULNERABILITIES.xlsx, TASKS.md, and MEMORY.md
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1242,6 +1242,90 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SEC-701</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>P2-4</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sample Dataset Secret and PII Exposure Prevention</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CWE-312</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Sample datasets or SQL seed scripts could accidentally bundle real production API keys, secrets, or customer PII.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>All demo entities utilize synthetic profiles with RFC 2606 reserved domains (.test, .demo); verified by automated regex secret scanning test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SEC-702</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>P2-4</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Production Data Pollution via Demo Bootstrap Execution</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CWE-284</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Automated demo seed execution could contaminate live production database tables if run outside demo environment.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Bootstrap service is strictly guarded behind DEMO_MODE=true in lifespan and implements database emptiness checks to prevent accidental execution.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(security): implement HS256 JWT authentication and require_role RBAC (P3-1)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Vulnerabilities" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vulnerabilities" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1326,6 +1326,90 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SEC-801</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>P3-1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>JWT Algorithm Confusion and None Algorithm Attack</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>CWE-345</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Forged JWT tokens signed with unexpected symmetric keys, public keys, or using alg=none could bypass signature verification and elevate privileges.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>decode_access_token explicitly specifies algorithms=["HS256"] and validates required iat/exp claims; verified by automated penetration test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SEC-802</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>P3-1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Privilege Escalation via Role Claim Manipulation and RBAC Boundary</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>CWE-269</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Malformed, synthetic, or unmapped role strings in JWT tokens could bypass access controls if authorization fallback defaults to permissive access.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Strict enum validation to RoleEnum rejects unmapped roles with HTTP 401; require_role enforces strict numerical hierarchy (viewer:1 &lt; agent:2 &lt; admin:3) defaulting unknown roles to level 0.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(auth): implement demo auth routes, token exchange, and profile endpoints (P3-2)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1410,6 +1410,90 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SEC-901</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>P3-2</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Production Exposure of Demo Token Generation Endpoint</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>CWE-284</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Exposing pre-signed JWT tokens for admin, agent, and viewer accounts without authentication could allow full system takeover in production.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>GET /api/v1/auth/demo-tokens is strictly guarded by DEMO_MODE=True and rejects calls in production/staging environments with HTTP 403 Forbidden; verified by automated penetration test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SEC-902</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>P3-2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Authentication Credential Enumeration via Asymmetric Feedback</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CWE-204</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Differentiating between invalid username and invalid password in login responses enables attackers to enumerate valid customer/staff email addresses.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>POST /api/v1/auth/login returns uniform HTTP 401 Unauthorized with generic "Invalid credentials" detail regardless of whether the user exists or password failed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(cache): implement Redis connection factory and fixed-window rate limiting middleware (P3-3)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1494,6 +1494,90 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SEC-1001</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>P3-3</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Fail-Closed Denial of Service on Cache Layer Outage</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>CWE-755</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Uncaught Redis connection or timeout exceptions in request middleware could fail closed, producing HTTP 500 errors across all API endpoints during a cache outage.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>RateLimitMiddleware implements resilient try/except blocks catching REDIS_EXCEPTIONS, logging structured warnings, and failing open to preserve application availability; verified by automated penetration test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SEC-1002</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>P3-3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Unbounded Redis Key Accumulation &amp; Memory Exhaustion</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CWE-770</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Creating rate limit keys for arbitrary client IP addresses without expiration could permanently consume Redis memory, triggering out-of-memory crashes.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Middleware applies an atomic EXPIRE of 60 seconds upon first INCR of each window key, ensuring automatic eviction and bounded memory consumption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(audit): implement AuditMiddleware and enforce pipeline ordering (P3-4)
- Implemented AuditMiddleware in backend/app/middleware/audit.py
- Intercepted all state-changing HTTP requests (POST, PUT, PATCH, DELETE) and logged immutable rows to audit_logs table
- Strictly excluded read-only requests (GET, HEAD, OPTIONS) to prevent table bloat (AC-069)
- Enforced complete middleware pipeline order: CORS (outermost) -> RequestId -> RateLimit -> Audit (innermost)
- Extracted actor UUID from Bearer token claims or defaulted to unauthenticated
- Extracted client IP and correlated request_id from headers/context
- Added resilient fail-safe error handling for audit database write failures (CWE-755)
- Added 6 comprehensive unit, integration, and security tests in tests/unit/test_audit_middleware.py (TC-128 to TC-133)
- Documented security vulnerabilities SEC-1101 and SEC-1102 in docs/SECURITY_VULNERABILITIES.xlsx
- Updated docs/TEST_CASES.xlsx, docs/TASKS.md, and docs/MEMORY.md
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vulnerabilities" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Vulnerabilities" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1578,6 +1578,90 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SEC-1101</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>P3-4</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Audit Log Injection &amp; Actor Spoofing via Malformed Headers</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>CWE-117</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Attacker injects falsified actor ID or client IP via manipulated Authorization or X-Forwarded-For headers to tamper with audit trails or frame legitimate users.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Actor identity is cryptographically validated using HS256 decode_access_token; untrusted tokens fallback to unauthenticated; IP header is parsed for first hop; writes are parameterized via SQLAlchemy ORM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SEC-1102</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>P3-4</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Denial of Service via Audit Store Exhaustion or Database Outage</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>CWE-755</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Database downtime, slow transaction locks, or high query volumes could cause audit logging failures that fail closed and crash customer-facing HTTP endpoints.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>AuditMiddleware encapsulates persistence in AUDIT_DB_EXCEPTIONS try/except, logging errors safely to system logs; rate limiting runs before audit logging to filter unauthenticated request floods.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(api): implement ticket and customer API contract and schemas (P4-1)
- Authoritative written API contract docs/API_CONTRACT.md defining routes, statuses, error envelopes, and RBAC rules
- Pydantic v2 schemas in backend/app/schemas/tickets.py and backend/app/schemas/customers.py
- Synchronized TypeScript type definitions in frontend/lib/types.ts
- Unit, validation, boundary, and security penetration test suite in tests/unit/test_schemas_contract.py (29 new tests, 162 total)
- Updated docs/TEST_CASES.xlsx (TC-134 to TC-162) and docs/SECURITY_VULNERABILITIES.xlsx (SEC-1201 to SEC-1204)
- Updated docs/TASKS.md and docs/MEMORY.md Honest Status
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1662,6 +1662,159 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SEC-1201</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>P4-1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Mass Assignment &amp; Parameter Injection in Ingestion Schemas</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>CWE-915</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Attackers injecting arbitrary parameters (e.g., status, assigned_to, is_admin) during public ticket ingestion or customer profile creation to bypass workflow stages or manipulate authorization.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Configured model_config = ConfigDict(extra="forbid") on TicketCreate, ReplyCreate, CustomerCreate, and CustomerMemoryCreate, causing Pydantic to actively reject unexpected fields with HTTP 422.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SEC-1202</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>P4-1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Denial of Service via Unbounded Ingestion Payload Memory Exhaustion</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>CWE-400</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Lack of strict upper bounds on request message bodies, subjects, and notes allows malicious actors to submit multi-megabyte payloads, causing memory exhaustion and API denial of service.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Enforced strict Pydantic Field boundary constraints (body &lt;= 50,000 chars, subject &lt;= 255 chars, notes &lt;= 5,000 chars); oversized requests are aborted before memory allocation or DB persistence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SEC-1203</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>P4-1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Prototype Pollution &amp; Object Attribute Injection Resistance</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>CWE-1321</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>JSON payloads containing dangerous keys like __proto__, constructor, or __class__ attempt to manipulate object properties or trigger runtime prototype pollution.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Strict Pydantic v2 schema validation with extra="forbid" explicitly validates and rejects special object keys, treating all properties as typed attributes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SEC-1204</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>P4-1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Cross-Site Scripting (XSS) &amp; Stored HTML Injection Containment</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>CWE-79</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Ingested ticket bodies and messages containing HTML/JS (&lt;script&gt;alert(1)&lt;/script&gt;) could lead to stored XSS if reflected or rendered unsanitized in the console.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Enforced N4 requirement treating ticket text strictly as untrusted raw string data; Pydantic preserves unicode without executing or stripping, and frontend interfaces mirror typed data strings without raw HTML rendering.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(api): implement support ticket API endpoints (P4-2)
- Ingestion route POST /api/v1/tickets with customer validation and atomic message creation
- Queue listing route GET /api/v1/tickets with multi-attribute filtering (status, severity, category, plan) and pagination
- Ticket dossier route GET /api/v1/tickets/{id} with conversation history and customer dossier
- Agent action routes POST /api/v1/tickets/{id}/reply and /request-info transitioning status to waiting_on_customer
- Policy and manual escalation route POST /api/v1/tickets/{id}/escalate with Escalation persistence
- RBAC protection requiring viewer role for read operations and agent role for state modifications
- Integration, boundary, and security test suite in tests/api/test_tickets.py (28 new tests, 190 total)
- Updated docs/TEST_CASES.xlsx (TC-163 to TC-190) and docs/SECURITY_VULNERABILITIES.xlsx (SEC-1301 to SEC-1304)
- Updated docs/TASKS.md and docs/MEMORY.md Honest Status
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1815,6 +1815,159 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SEC-1301</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>P4-2</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Privilege Escalation on Ticket Modification and Escalation Routes</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>CWE-285</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Unprivileged viewer roles attempting to dispatch replies, request customer clarifications, or escalate tickets to manipulate support workflows.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Enforced require_role(RoleEnum.AGENT) dependency on POST /reply, POST /request-info, and POST /escalate routes; unauthorized callers receive HTTP 403 Forbidden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SEC-1302</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>P4-2</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Insecure Direct Object Reference &amp; Customer Ingestion Spoofing</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>CWE-639</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Public ticket ingestion specifying arbitrary non-existent or synthetic customer IDs creating orphaned or spoofed ticket records.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>create_ticket performs mandatory customer existence check via CustomerRepository.get(customer_id) within the transaction; returns HTTP 404 and rolls back if customer does not exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SEC-1303</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>P4-2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SQL Injection in Multi-Parameter Ticket Queue Filters</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>CWE-89</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Attackers injecting SQL fragments via status, severity, category, plan, or customer_id query parameters to dump ticket databases or bypass RBAC filters.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Strict enum parsing in Pydantic/FastAPI and query parameterization through SQLAlchemy ORM expressions (Ticket.status == status, Ticket.customer_id == customer_id).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SEC-1304</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>P4-2</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Stored Cross-Site Scripting (XSS) in Omnichannel Ticket Messages</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>CWE-79</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Inbound ticket bodies and messages containing embedded HTML or JavaScript tags (&lt;script&gt;alert(1)&lt;/script&gt;) triggering stored XSS in agent consoles.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Implemented N4 requirement isolating ticket text strictly as untrusted UTF-8 data; inputs are preserved verbatim without HTML rendering or execution hazards.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(api): implement customer API endpoints and secret scrubbing (P4-3)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1968,6 +1968,174 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SEC-1401</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>P4-3</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Automated Secret and Credential Scrubbing in Customer Memory</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>CWE-200</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Fixed &amp; Verified</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Customer support interactions may inadvertently transmit credit card numbers, API keys, or raw passwords into persistent memory notes.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Implemented scrub_secrets() with regex redaction replacing card numbers, API tokens, and passwords with [REDACTED] prior to DB persistence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SEC-1402</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>P4-3</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Customer Tenant Context &amp; Resource Isolation Boundary</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>CWE-639</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Dossier lookup could inadvertently query or expose tickets, subscriptions, or workspaces across tenant boundaries (IDOR).</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Strictly filtered all repository queries by customer_id matching the authenticated context; verified zero cross-customer data leakage (AC-023).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SEC-1403</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>P4-3</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Enum Parameter Validation Preventing Query Injection</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>CWE-89</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>SQL injection attempts in plan query parameter on customer list endpoint.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Enforced FastAPI CustomerPlanEnum type annotation and SQLAlchemy parameterized queries; invalid inputs rejected with HTTP 422.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SEC-1404</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>P4-3</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Role-Based Privilege Escalation on Memory &amp; Customer Creation</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>CWE-285</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Viewer role users attempting to create customer profiles or mutate customer institutional memory.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Applied require_role(RoleEnum.AGENT) dependency to POST /customers and POST /customers/{id}/memory returning HTTP 403 Forbidden.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(rag): implement knowledge article loading and heading-based chunking (P5-1)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2136,6 +2136,174 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SEC-1501</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>P5-1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Path Traversal Containment in Markdown Knowledge Loader</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>CWE-22</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Article file loader could allow reading arbitrary files on the filesystem if unvalidated paths are accepted.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Enforced strict file existence checks, markdown extension matching, and mandatory YAML front-matter header verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SEC-1502</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>P5-1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Stored Script / Cross-Site Scripting Encapsulation in Chunks</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>CWE-79</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Malicious HTML or script tags inside knowledge base articles could execute in agent console web UI.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Chunks parse markdown strictly as untrusted raw text data without executing markup; frontend renders text nodes safely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SEC-1503</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>P5-1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ReDoS &amp; Resource Exhaustion Defense in Heading Parser</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>CWE-400</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Crafted markdown with repeated heading markers could trigger catastrophic regex backtracking in section splitters.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Implemented anchored non-backtracking regex patterns evaluated line-by-line in linear O(N) execution time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SEC-1504</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>P5-1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Secret &amp; PII Elimination from Static Knowledge Base Articles</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>CWE-200</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Committed sample knowledge base articles or generated chunks could inadvertently leak sensitive API keys or credentials.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Automated regex penetration test in CI verifies zero payment cards, API tokens, or credentials exist in knowledge base files.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(rag): implement vector store and fake embeddings (P5-2)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2304,6 +2304,174 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SEC-1601</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>P5-2</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Command / SQL Injection Neutralization in Vector Search Queries</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>CWE-89</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Adversarial input payloads containing SQL, NoSQL, or command strings passed as search queries to vector search endpoints.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Dense query embedding hashes raw strings purely into mathematical vector coordinates; queries never reach SQL evaluation or dynamic execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SEC-1602</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>P5-2</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Denial of Service via Massive Document Embedding (ReDoS / Memory Exhaustion)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>CWE-400</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Massive text inputs (50,000+ characters) supplied to embedding algorithms causing memory spikes or CPU exhaustion.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Linear-time tokenization and MD5 digest extraction bound vector creation to O(N) single-pass computation with strict L2-normalization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SEC-1603</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>P5-2</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Metadata Injection &amp; Prototype Pollution Containment in Vector Documents</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CWE-1321</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Malicious vector document metadata dictionaries containing special keys (e.g. __proto__, constructor) attempting object pollution.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Isolated Python dictionaries cloned via dict(metadata) avoiding runtime attribute pollution; verified by test_security_metadata_isolation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SEC-1604</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>P5-2</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Offline Isolation &amp; Zero Data Leakage for Vector Store Credentials</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>CWE-200</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Third-party cloud vector stores requiring external API keys leaking secrets or failing during air-gapped demo runs.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Default configuration operates with zero-cloud InMemoryVectorStore and FakeEmbeddings without external network requests or keys.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(rag): implement hybrid retriever with BM25, RRF, and caching (P5-3)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2472,6 +2472,217 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SEC-1701</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>P5-3</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CRLF Injection and Cache Key Poisoning in Short-Term Memory</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>CWE-93</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Unsanitized search queries containing carriage returns and line feeds (CRLF) attempt Redis protocol manipulation or cache key collision/poisoning.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Query strings are stripped of CRLF characters (re.sub(r"[
+]+", " ", clean_query)[:256]) before cache key construction. Verified by test_security_cache_key_poisoning_containment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SEC-1702</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>P5-3</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Algorithmic Complexity and Query Denial of Service (ReDoS / Memory Exhaustion)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>CWE-1333</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Massive adversarial query strings (50,000+ characters) or repetitive regular expression patterns targeting the query tokenizer and BM25 scorer causing high CPU utilization or thread starvation.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Inputs to _tokenize() are capped at 50,000 characters and tokenized using non-backtracking linear word boundaries (word characters). Verified by test_security_redos_query_safety.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SEC-1703</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>P5-3</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Stored and Reflected Cross-Site Scripting (XSS) in Evidence Snippets</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>CWE-79</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Markdown articles or query payloads containing script tags (&lt;script&gt;alert(1)&lt;/script&gt;) attempting stored or reflected XSS execution in downstream web frontends.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>The retriever treats all article content, headings, and snippets as strict immutable string literals, returning typed evidence dictionaries without HTML/JS evaluation. Verified by test_security_xss_in_evidence_snippet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SEC-1704</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>P5-3</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Query Injection &amp; Protocol Escape in Hybrid Retrieval Backends</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>CWE-89</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>SQL and NoSQL injection payloads in query parameters attempt interpreter breakout, data dumping, or backend vector store manipulation.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Dense retrieval operates via fixed vector dimension hashing and cosine similarity; sparse retrieval operates via in-memory inverted token frequencies (BM25Okapi). No raw query strings are interpreted by an SQL/NoSQL engine. Verified by test_security_sql_and_nosql_injection_query_containment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SEC-1705</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>P5-3</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Denial of Service via Redis Cache Outage / Unhandled Exceptions</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>CWE-755</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Unhandled connection errors, timeouts, or network partitions in the short-term Redis cache tier crashing the RAG retrieval pipeline and blocking support ticket processing.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>All cache operations catch REDIS_EXCEPTIONS and degrade gracefully to live retrieval, logging a warning while preserving continuous system availability. Verified by test_redis_graceful_degradation_on_error.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(rag): implement ingest command and knowledge api (P5-4)
</commit_message>
<xml_diff>
--- a/docs/SECURITY_VULNERABILITIES.xlsx
+++ b/docs/SECURITY_VULNERABILITIES.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2683,6 +2683,216 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SEC-1801</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>P5-4</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Administrative Re-index RBAC Escalation &amp; DoS Defense</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>CWE-285</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Unauthenticated or non-admin users attempting to invoke POST /api/v1/knowledge/reindex, which wipes and rebuilds vector store collections.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Strict role-based authorization enforced via require_role(RoleEnum.ADMIN). Viewers and agents receive 403 Forbidden. Verified by test_knowledge_reindex_as_viewer_forbidden and test_knowledge_reindex_as_agent_forbidden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SEC-1802</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>P5-4</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Directory Path Traversal in Knowledge Article Lookup</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>CWE-22</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Arbitrary file disclosure via directory traversal sequences (e.g. ../../etc/passwd) in GET /api/v1/knowledge/articles/{id_or_slug}.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Explicit path traversal filter rejecting dot-dot sequences and directory separators, combined with memory-indexed article document lookup. Verified by test_security_path_traversal_in_article_endpoint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SEC-1803</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>P5-4</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Query Injection Neutralization in Knowledge Search Payload</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>CWE-89</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>SQL/NoSQL injection payloads in POST /api/v1/knowledge/search query attribute attempting database breakout.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Queries are strictly processed through offline FakeEmbeddings vector hashing and BM25 token frequencies without dynamic SQL/NoSQL compilation. Verified by test_security_sql_injection_in_search_query.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SEC-1804</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>P5-4</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Denial of Service via Unbounded Search Bounds and Modes</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>CWE-400</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Excessive resource consumption from massive queries, negative or unbounded top_k limits, or invalid search modes.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>KnowledgeSearchRequest schema enforces max_length=2000, non-blank validator, top_k bounds [1, 20], and mode regex validation. Verified by test_knowledge_search_invalid_top_k_bounds and test_knowledge_search_invalid_mode_rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SEC-1805</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>P5-4</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Stored &amp; Reflected Cross-Site Scripting (XSS) in Query and Article Dossier</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>CWE-79</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Protected</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Embedded HTML or JavaScript tags in search queries or markdown articles attempting stored/reflected XSS.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>All article content and snippet text are handled as immutable string primitives within typed JSON envelopes without HTML evaluation. Verified by test_security_xss_payload_in_query.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>